<commit_message>
Update internal student template and import instructions; enhance OJT export functionality
</commit_message>
<xml_diff>
--- a/BioTern/assets/Internal Students Template.xlsx
+++ b/BioTern/assets/Internal Students Template.xlsx
@@ -1,13 +1,20 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <sheets>
-    <sheet name="Internal Students" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>BioTern</Application>
+</Properties>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>BioTern</dc:creator>
+  <cp:lastModifiedBy>BioTern</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-05-01T00:00:00Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-05-01T00:00:00Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <fonts count="2">
     <font>
@@ -73,22 +80,27 @@
 </styleSheet>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Internal Students" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="2" width="16" customWidth="1"/>
-    <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="48" customWidth="1"/>
-    <col min="7" max="7" width="72" customWidth="1"/>
-    <col min="8" max="8" width="34" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
-    <col min="10" max="10" width="38" customWidth="1"/>
-    <col min="11" max="11" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="22" customWidth="1"/>
+    <col min="5" max="5" width="34" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="14" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -99,56 +111,41 @@
       </c>
       <c r="B1" t="inlineStr" s="1">
         <is>
-          <t>school_year</t>
+          <t>last_name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr" s="1">
         <is>
-          <t>STUDENT NAME</t>
+          <t>first_name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr" s="1">
         <is>
-          <t>CONTACT NO.</t>
+          <t>middle_name</t>
         </is>
       </c>
       <c r="E1" t="inlineStr" s="1">
         <is>
-          <t>SECTION</t>
+          <t>email</t>
         </is>
       </c>
       <c r="F1" t="inlineStr" s="1">
         <is>
-          <t>COMPANY</t>
+          <t>course_id</t>
         </is>
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t>ADDRESS</t>
+          <t>section_id</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
-          <t>SUPERVISOR NAME</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr" s="1">
-        <is>
-          <t>POSITION</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr" s="1">
-        <is>
-          <t>COMPANY REPRESENTATIVE</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr" s="1">
-        <is>
-          <t>STATUS</t>
+          <t>password</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K1"/>
+  <autoFilter ref="A1:H1"/>
 </worksheet>
 </file>
</xml_diff>